<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.002-01 Le cheval et le pont
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.002-01.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.002-01.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine après gâteaux, carton de céréales</t>
+          <t>cuisine après gâteaux, carton de céréales, plaque, beurre, farine sur les manches</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut que le cheval de bois traverse un pont en carton. Il propose. Victorina dit non, puis je regarde, puis plus tard. Nino accepte. Le pont se plie, il l'aplatit. Le cheval passe. Un mouton s'approche.</t>
+          <t>La plaque de gâteaux fume. Sur le bord, un éclat de plaque luit. Farine sur les manches. Nino veut le cheval sur le pont, maintenant, avec Victorina. Il tend trop vite : elle dit non, le pont se plie. Sourire parti. Papa à sa hauteur. Il refuse de foncer, attend son silence, dit d'accord. Merci vécu. Le cheval glisse. Il veut sa main : elle ne bouge pas. Il observe, retrouve l'éclat. Un éclat de plaque reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>De la farine blanche dort sur les manches de papa. La plaque de gâteaux refroidit. Ça sent le beurre encore chaud. Une miette sucrée colle au bois. Un carton de céréales est à plat. Des lettres bleues restent dessus. Nino l'a plié en pont. Un cheval de bois attend. Sa crinière est peinte en brun. Un mouton de bois aussi. Tu as vu la farine, Nino ? Oui, maman. Sur les manches. Les gâteaux attendent un peu. On reste par terre. Le cheval va sur le pont. Jusqu'à l'autre côté ? Oui. Le mouton après. En ce moment, Nino pose le pont. Le carton est un peu rêche. Il appuie les deux bords. Maman ouvre la porte. Victorina arrive. Elle a des chaussettes jaunes. Tu viens ? Non. Nino regarde papa. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Nino pousse le cheval. Les sabots glissent un peu. Le pont se plie au milieu. Oh. Tu as vu le pli, Nino ? Oui. Nino aplatit le carton. Il passe la main dessus. Le pont redevient droit. Tu proposes encore, tout doux ? Plus tard, tu viens ? Je regarde. Regarder, c'est une réponse.</t>
+          <t>La plaque de gâteaux fume un peu. Ça sent le beurre, dans la cuisine. Sur le bord, un éclat de plaque luit. Il brille, papa. Tu le vois, sur la plaque ? Nino touche l'éclat de plaque, un instant. Le métal est tiède, un peu gras. Elle est chaude. Les gâteaux attendent un peu. On reste par terre. De la farine blanche dort sur les manches. Sur tes manches, papa. Oui, un peu. Un carton de céréales est à plat. Des lettres bleues restent dessus. Je le plie en pont. Un pont, par terre ? Oui, maman. Nino plie le carton, deux bords. Un petit cheval peint attend. Sa crinière est brune, un peu raide. Le cheval va sur le pont. Jusqu'à l'autre côté ? Oui. Un mouton peint attend aussi. Le mouton après. En ce moment, Nino pose le pont. Le carton est rêche, un peu chaud. Il appuie les deux bords. Tu restes près de nous ? Oui, maman. Maman ouvre la porte. Victorina arrive. Elle a des chaussettes jaunes. Tu viens ? Non. Nino tend la main trop vite. Il pousse le cheval d'un coup. Tu le pousses, Nino ? Les sabots glissent un peu. Le pont se plie au milieu. Oh. Tu as vu le carton, Nino ? Oui. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu viens, maintenant ! Non. Victorina recule d'un pas. Ses épaules restent près de la porte. Je le prends ! Le pont s'est plié. Tu le vois, Nino ? Les épaules de Nino tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>De la farine blanche dort sur les manches de papa. La plaque de gâteaux refroidit. Ça sent le beurre encore chaud. Une miette sucrée colle au bois. Un carton de céréales est à plat. Des lettres bleues restent dessus. Nino l'a plié en pont. Un cheval de bois attend. Sa crinière est peinte en brun. Un mouton de bois aussi. Tu as vu la farine, Nino ? Oui, maman. Sur les manches. Les gâteaux attendent un peu. On reste par terre. Le cheval va sur le pont. Jusqu'à l'autre côté ? Oui. Le mouton après. En ce moment, Nino pose le pont. Le carton est un peu rêche. Il appuie les deux bords. Maman ouvre la porte. Victorina arrive. Elle a des chaussettes jaunes. Tu viens ? Non. Nino regarde papa. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Nino pousse le cheval. Les sabots glissent un peu. Le pont se plie au milieu. Oh. Tu as vu le pli, Nino ? Oui. Nino aplatit le carton. Il passe la main dessus. Le pont redevient droit. Tu proposes encore, tout doux ? Plus tard, tu viens ? Je regarde. Regarder, c'est une réponse.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La plaque de gâteaux fume un peu. Ça sent le beurre, dans la cuisine. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de plaque&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur la plaque ? Nino touche l'éclat de plaque, un instant. Le métal est tiède, un peu gras. Elle est chaude. Les gâteaux attendent un peu. On reste par terre. De la farine blanche dort sur les manches. Sur tes manches, papa. Oui, un peu. Un carton de céréales est à plat. Des lettres bleues restent dessus. Je le plie en pont. Un pont, par terre ? Oui, maman. Nino plie le carton, deux bords. Un petit cheval peint attend. Sa crinière est brune, un peu raide. Le cheval va sur le pont. Jusqu'à l'autre côté ? Oui. Un mouton peint attend aussi. Le mouton après. En ce moment, Nino pose le pont. Le carton est rêche, un peu chaud. Il appuie les deux bords. Tu restes près de nous ? Oui, maman. Maman ouvre la porte. Victorina arrive. Elle a des chaussettes jaunes. Tu viens ? Non. Nino tend la main trop vite. Il pousse le cheval d'un coup. Tu le pousses, Nino ? Les sabots glissent un peu. Le pont se plie au milieu. Oh. Tu as vu le carton, Nino ? Oui. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu viens, maintenant ! Non. Victorina recule d'un pas. Ses épaules restent près de la porte. Je le prends ! Le pont s'est plié. Tu le vois, Nino ? Les épaules de Nino tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom est dans le salon. Les cubes sont par terre. Maman ouvre la porte. Ava arrive. Tom veut jouer. Il va &lt;emphasis&gt;proposer&lt;/emphasis&gt; un jeu. Tom dit : tu viens ? Ava dit : non. Tom regarde maman. Maman dit : on peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Tom dit : d'accord. Il construit une tour. Ava s'assoit près du canapé. Elle regarde. Tom laisse Ava à sa place. Il propose encore, tout doux. Tom dit : plus tard, tu viens ? Ava dit : je regarde. Maman sourit. Maman dit : regarder, c'est une réponse. On peut accepter plusieurs réponses. Tom pose un cube rouge. Il pose un cube bleu. La tour grandit. Ava avance un peu. Elle ne touche pas. C'est bien. Tom dit : tu veux un cube ? Ava dit : plus tard. Tom dit : d'accord. Il continue. Maman chante tout bas. La tour tombe. Tom rit. Il va proposer : on recommence. Ava hoche la tête. Elle vient. Elle pose un cube jaune. Puis elle s'arrête. Tom accepte. Ils restent près des cubes. Maman dit : tu as su proposer. Tu as su accepter. Plusieurs réponses sont possibles. Non. Regarder. Plus tard. Oui, un peu. Tout ça va.&lt;/slow&gt; [pause]</t>
+          <t>La plaque de gâteaux fume un peu. Ça sent le beurre, dans la cuisine. Sur le bord, un &lt;emphasis&gt;éclat de plaque&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur la plaque ? Nino touche l'éclat de plaque, un instant. Le métal est tiède, un peu gras. Elle est chaude. Les gâteaux attendent un peu. On reste par terre. De la farine blanche dort sur les manches. Sur tes manches, papa. Oui, un peu. Un carton de céréales est à plat. Des lettres bleues restent dessus. Je le plie en pont. Un pont, par terre ? Oui, maman. Nino plie le carton, deux bords. Un petit cheval peint attend. Sa crinière est brune, un peu raide. Le cheval va sur le pont. Jusqu'à l'autre côté ? Oui. Un mouton peint attend aussi. Le mouton après. En ce moment, Nino pose le pont. Le carton est rêche, un peu chaud. Il appuie les deux bords. Tu restes près de nous ? Oui, maman. Maman ouvre la porte. Victorina arrive. Elle a des chaussettes jaunes. Tu viens ? Non. Nino tend la main trop vite. Il pousse le cheval d'un coup. Tu le pousses, Nino ? Les sabots glissent un peu. Le pont se plie au milieu. Oh. Tu as vu le carton, Nino ? Oui. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu viens, maintenant ! Non. Victorina recule d'un pas. Ses épaules restent près de la porte. Je le prends ! Le pont s'est plié. Tu le vois, Nino ? Les épaules de Nino tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>éclat de plaque</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,59 +1324,71 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_cheval_et_victorina_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|De la farine blanche dort sur les manches de papa.
-narrateur|La plaque de gâteaux refroidit.
-narrateur|Ça sent le beurre encore chaud.
-narrateur|Une miette sucrée colle au bois.
+          <t>narrateur|La plaque de gâteaux fume un peu.
+narrateur|Ça sent le beurre, dans la cuisine.
+narrateur|Sur le bord, un éclat de plaque luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur la plaque ?
+narrateur|Nino touche l'éclat de plaque, un instant.
+narrateur|Le métal est tiède, un peu gras.
+enfant-m|Elle est chaude.
+maman|Les gâteaux attendent un peu.
+papa|On reste par terre.
+narrateur|De la farine blanche dort sur les manches.
+enfant-m|Sur tes manches, papa.
+papa|Oui, un peu.
 narrateur|Un carton de céréales est à plat.
 narrateur|Des lettres bleues restent dessus.
-narrateur|Nino l'a plié en pont.
-narrateur|Un cheval de bois attend.
-narrateur|Sa crinière est peinte en brun.
-narrateur|Un mouton de bois aussi.
-maman|Tu as vu la farine, Nino ?
+enfant-m|Je le plie en pont.
+maman|Un pont, par terre ?
 enfant-m|Oui, maman.
-enfant-m|Sur les manches.
-papa|Les gâteaux attendent un peu.
-papa|On reste par terre.
+narrateur|Nino plie le carton, deux bords.
+narrateur|Un petit cheval peint attend.
+narrateur|Sa crinière est brune, un peu raide.
 enfant-m|Le cheval va sur le pont.
 maman|Jusqu'à l'autre côté ?
 enfant-m|Oui.
+narrateur|Un mouton peint attend aussi.
 enfant-m|Le mouton après.
 narrateur|En ce moment, Nino pose le pont.
-narrateur|Le carton est un peu rêche.
+narrateur|Le carton est rêche, un peu chaud.
 narrateur|Il appuie les deux bords.
+maman|Tu restes près de nous ?
+enfant-m|Oui, maman.
 narrateur|Maman ouvre la porte.
 narrateur|Victorina arrive.
 narrateur|Elle a des chaussettes jaunes.
 enfant-m|Tu viens ?
 copine|Non.
-narrateur|Nino regarde papa.
-papa|On peut proposer.
-maman|On peut accepter plusieurs réponses.
-papa|Oui.
-papa|Non.
-papa|Regarder.
-papa|Plus tard.
-enfant-m|D'accord.
-narrateur|Nino pousse le cheval.
+narrateur|Nino tend la main trop vite.
+narrateur|Il pousse le cheval d'un coup.
+papa|Tu le pousses, Nino ?
 narrateur|Les sabots glissent un peu.
 narrateur|Le pont se plie au milieu.
 enfant-m|Oh.
-papa|Tu as vu le pli, Nino ?
+papa|Tu as vu le carton, Nino ?
 enfant-m|Oui.
-narrateur|Nino aplatit le carton.
-narrateur|Il passe la main dessus.
-narrateur|Le pont redevient droit.
-maman|Tu proposes encore, tout doux ?
-enfant-m|Plus tard, tu viens ?
-copine|Je regarde.
-papa|Regarder, c'est une réponse.</t>
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Tu viens, maintenant !
+copine|Non.
+narrateur|Victorina recule d'un pas.
+narrateur|Ses épaules restent près de la porte.
+enfant-m|Je le prends !
+maman|Le pont s'est plié.
+papa|Tu le vois, Nino ?
+narrateur|Les épaules de Nino tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1413,12 +1425,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino invite Victorina. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino invite &lt;emphasis level="moderate"&gt;Victorina&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom invite Ava. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino invite &lt;emphasis&gt;Victorina&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1481,7 +1493,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1489,10 +1501,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1507,34 +1519,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Victorina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1543,13 +1559,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1559,7 +1575,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nino_invite_sans_forcer; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1592,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino a su proposer. Il accepte plusieurs réponses. D'accord. Victorina s'assoit près du buffet. Elle regarde le cheval. Nino pousse encore. Les sabots tapent le carton. Tu as entendu les sabots ? Oui, papa. Tu veux le mouton ? Plus tard. D'accord. Plusieurs réponses sont possibles. Le cheval avance au milieu. Le pont tient. Tu as aplati le pli. Oui. Une miette tombe près du pont. Nino la pousse du doigt. Victorina avance un peu. Elle reste à regarder. C'est bien. Le beurre sent encore.</t>
+          <t>Nino avance trop vite vers le pont. Tu viens, maintenant ! Sa voix se mélange au carton. Oh. Victorina reste près de la porte. Il refuse de foncer. Nino referme la main. Tu veux venir près du pont ? Papa s'accroupit à la même hauteur. Nino pose un genou près du carton. Tu regardes ? Victorina ne dit rien. Elle reste un moment, les mains collées. Plus tard, tu viens ? Je regarde. D'accord. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Nino aplatit le carton, sans le jeter. Le pont redevient droit. Il tient. Le cheval est là. Nino pose le cheval près du bord. Les sabots tapent le carton. Tu as entendu les sabots ? Oui, papa. Tu veux le mouton ? Plus tard. D'accord. Victorina s'assoit près du buffet. Elle regarde le cheval. Il avance ? Un peu. Une miette tombe près du pont. Nino la pousse du doigt.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino a su proposer. Il accepte plusieurs réponses. D'accord. Victorina s'assoit près du buffet. Elle regarde le cheval. Nino pousse encore. Les sabots tapent le carton. Tu as entendu les sabots ? Oui, papa. Tu veux le mouton ? Plus tard. D'accord. Plusieurs réponses sont possibles. Le cheval avance au milieu. Le pont tient. Tu as aplati le pli. Oui. Une miette tombe près du pont. Nino la pousse du doigt. Victorina avance un peu. Elle reste à regarder. C'est bien. Le beurre sent encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino avance trop vite vers le pont. Tu viens, maintenant ! Sa voix se mélange au carton. Oh. Victorina reste près de la porte. Il refuse de foncer. Nino referme la main. Tu veux venir près du pont ? Papa s'accroupit à la même hauteur. Nino pose un genou près du carton. Tu regardes ? Victorina ne dit rien. Elle reste un moment, les mains collées. Plus tard, tu viens ? Je regarde. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Nino aplatit le carton, sans le jeter. Le pont redevient droit. Il tient. Le cheval est là. Nino pose le cheval près du bord. Les sabots tapent le carton. Tu as entendu les sabots ? Oui, papa. Tu veux le mouton ? Plus tard. D'accord. Victorina s'assoit près du buffet. Elle regarde le cheval. Il avance ? Un peu. Une miette tombe près du pont. Nino la pousse du doigt.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom a su &lt;emphasis&gt;proposer&lt;/emphasis&gt;. Ava a dit non, puis regarder. Tom a pu accepter plusieurs réponses.&lt;/slow&gt; [pause]</t>
+          <t>Nino avance trop vite vers le pont. Tu viens, maintenant ! Sa voix se mélange au carton. Oh. Victorina reste près de la porte. Il refuse de foncer. Nino referme la main. Tu veux venir près du pont ? Papa s'accroupit à la même hauteur. Nino pose un genou près du carton. Tu regardes ? Victorina ne dit rien. Elle reste un moment, les mains collées. Plus tard, tu viens ? Je regarde. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Nino aplatit le carton, sans le jeter. Le pont redevient droit. Il tient. Le cheval est là. Nino pose le cheval près du bord. Les sabots tapent le carton. Tu as entendu les sabots ? Oui, papa. Tu veux le mouton ? Plus tard. D'accord. Victorina s'assoit près du buffet. Elle regarde le cheval. Il avance ? Un peu. Une miette tombe près du pont. Nino la pousse du doigt. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1649,18 +1665,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1683,7 +1699,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1693,20 +1709,20 @@
         <v>450</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1715,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1727,43 +1743,59 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=il_attend_le_silence_puis_dit_d_accord; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino a su proposer.
-narrateur|Il accepte plusieurs réponses.
+          <t>narrateur|Nino avance trop vite vers le pont.
+enfant-m|Tu viens, maintenant !
+narrateur|Sa voix se mélange au carton.
+enfant-m|Oh.
+narrateur|Victorina reste près de la porte.
+narrateur|Il refuse de foncer.
+narrateur|Nino referme la main.
+papa|Tu veux venir près du pont ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Nino pose un genou près du carton.
+enfant-m|Tu regardes ?
+narrateur|Victorina ne dit rien.
+narrateur|Elle reste un moment, les mains collées.
+enfant-m|Plus tard, tu viens ?
+copine|Je regarde.
 enfant-m|D'accord.
-narrateur|Victorina s'assoit près du buffet.
-narrateur|Elle regarde le cheval.
-narrateur|Nino pousse encore.
+papa|Merci, Nino.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-m|Un peu, maman.
+narrateur|Nino aplatit le carton, sans le jeter.
+narrateur|Le pont redevient droit.
+enfant-m|Il tient.
+maman|Le cheval est là.
+narrateur|Nino pose le cheval près du bord.
 narrateur|Les sabots tapent le carton.
 papa|Tu as entendu les sabots ?
 enfant-m|Oui, papa.
 enfant-m|Tu veux le mouton ?
 copine|Plus tard.
 enfant-m|D'accord.
-maman|Plusieurs réponses sont possibles.
-narrateur|Le cheval avance au milieu.
-narrateur|Le pont tient.
-papa|Tu as aplati le pli.
-enfant-m|Oui.
+narrateur|Victorina s'assoit près du buffet.
+narrateur|Elle regarde le cheval.
+papa|Il avance ?
+enfant-m|Un peu.
 narrateur|Une miette tombe près du pont.
-narrateur|Nino la pousse du doigt.
-narrateur|Victorina avance un peu.
-narrateur|Elle reste à regarder.
-maman|C'est bien.
-maman|Le beurre sent encore.</t>
+narrateur|Nino la pousse du doigt.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>bois</t>
+          <t>cheval,carton</t>
         </is>
       </c>
     </row>
@@ -1790,17 +1822,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Victorina tend la main. Elle pose le mouton près du pont. Merci. Tu as accepté, Nino ? Oui, papa. Bravo. Le cheval finit le pont. Il arrive de l'autre côté. Il est passé. Le mouton aussi, après. Clip, clop. Clip, clop. Les gâteaux sont tièdes, maintenant. On range le pont ? Oui. Nino plie le carton. Les lettres bleues se plient aussi. Victorina pose le cheval. Le mouton reste près d'elle. Tu as fini le pont ? Oui, papa.</t>
+          <t>Nino pousse le cheval trop vite. Tu marches jusqu'au bout ! Le cheval glisse au milieu. Le carton se lève d'un côté. Oh. Le cheval penche vers le sol. Je le prends ! Nino avance la main vers Victorina. Tu l'attends, Nino ? Victorina ne bouge pas. Ses mains restent sur ses genoux. Attends, je regarde. Nino s'arrête net. Papa attend, sans parler. Je regarde. Nino observe la plaque, écoute la cuisine. Sur le bord, un éclat de plaque luit. Là, près des gâteaux. Nino tient le cheval des deux mains. Le carton est rêche, un peu tiède. Il est tiède, papa. Tu le portes jusqu'au bout ? Oui, papa. On avance ? Oui, maman. Nino pose le cheval au début. Il pousse, très peu. Il passe. Le mouton aussi, après. Victorina tend la main. Elle pose le mouton près du pont. Tu le tiens, Nino ? Oui. Les sabots tapent, puis se taisent. Le cheval arrive de l'autre côté. Il est passé. Les gâteaux sont tièdes. On plie le pont ? Oui. Nino plie le carton. Les lettres bleues se plient aussi.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Victorina tend la main. Elle pose le mouton près du pont. Merci. Tu as accepté, Nino ? Oui, papa. Bravo. Le cheval finit le pont. Il arrive de l'autre côté. Il est passé. Le mouton aussi, après. Clip, clop. Clip, clop. Les gâteaux sont tièdes, maintenant. On range le pont ? Oui. Nino plie le carton. Les lettres bleues se plient aussi. Victorina pose le cheval. Le mouton reste près d'elle. Tu as fini le pont ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino pousse le cheval trop vite. Tu marches jusqu'au bout ! Le cheval glisse au milieu. Le carton se lève d'un côté. Oh. Le cheval penche vers le sol. Je le prends ! Nino avance la main vers Victorina. Tu l'attends, Nino ? Victorina ne bouge pas. Ses mains restent sur ses genoux. Attends, je regarde. Nino s'arrête net. Papa attend, sans parler. Je regarde. Nino observe la plaque, écoute la cuisine. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de plaque&lt;/emphasis&gt; luit. Là, près des gâteaux. Nino tient le cheval des deux mains. Le carton est rêche, un peu tiède. Il est tiède, papa. Tu le portes jusqu'au bout ? Oui, papa. On avance ? Oui, maman. Nino pose le cheval au début. Il pousse, très peu. Il passe. Le mouton aussi, après. Victorina tend la main. Elle pose le mouton près du pont. Tu le tiens, Nino ? Oui. Les sabots tapent, puis se taisent. Le cheval arrive de l'autre côté. Il est passé. Les gâteaux sont tièdes. On plie le pont ? Oui. Nino plie le carton. Les lettres bleues se plient aussi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Maman dit : on range. Tom met un cube dans la boîte. Ava met le cube jaune. Ils se disent merci.&lt;/slow&gt; [pause]</t>
+          <t>Nino pousse le cheval trop vite. Tu marches jusqu'au bout ! Le cheval glisse au milieu. Le carton se lève d'un côté. Oh. Le cheval penche vers le sol. Je le prends ! Nino avance la main vers Victorina. Tu l'attends, Nino ? Victorina ne bouge pas. Ses mains restent sur ses genoux. Attends, je regarde. Nino s'arrête net. Papa attend, sans parler. Je regarde. Nino observe la plaque, écoute la cuisine. Sur le bord, un &lt;emphasis&gt;éclat de plaque&lt;/emphasis&gt; luit. Là, près des gâteaux. Nino tient le cheval des deux mains. Le carton est rêche, un peu tiède. Il est tiède, papa. Tu le portes jusqu'au bout ? Oui, papa. On avance ? Oui, maman. Nino pose le cheval au début. Il pousse, très peu. Il passe. Le mouton aussi, après. Victorina tend la main. Elle pose le mouton près du pont. Tu le tiens, Nino ? Oui. Les sabots tapent, puis se taisent. Le cheval arrive de l'autre côté. Il est passé. Les gâteaux sont tièdes. On plie le pont ? Oui. Nino plie le carton. Les lettres bleues se plient aussi. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1847,18 +1879,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1879,28 +1911,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plaque</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1909,10 +1945,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1921,37 +1957,61 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_forcer_la_main_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Victorina tend la main.
+          <t>narrateur|Nino pousse le cheval trop vite.
+enfant-m|Tu marches jusqu'au bout !
+narrateur|Le cheval glisse au milieu.
+narrateur|Le carton se lève d'un côté.
+enfant-m|Oh.
+narrateur|Le cheval penche vers le sol.
+enfant-m|Je le prends !
+narrateur|Nino avance la main vers Victorina.
+papa|Tu l'attends, Nino ?
+narrateur|Victorina ne bouge pas.
+narrateur|Ses mains restent sur ses genoux.
+enfant-m|Attends, je regarde.
+narrateur|Nino s'arrête net.
+narrateur|Papa attend, sans parler.
+enfant-m|Je regarde.
+narrateur|Nino observe la plaque, écoute la cuisine.
+narrateur|Sur le bord, un éclat de plaque luit.
+enfant-m|Là, près des gâteaux.
+narrateur|Nino tient le cheval des deux mains.
+narrateur|Le carton est rêche, un peu tiède.
+enfant-m|Il est tiède, papa.
+papa|Tu le portes jusqu'au bout ?
+enfant-m|Oui, papa.
+maman|On avance ?
+enfant-m|Oui, maman.
+narrateur|Nino pose le cheval au début.
+narrateur|Il pousse, très peu.
+enfant-m|Il passe.
+copine|Le mouton aussi, après.
+narrateur|Victorina tend la main.
 narrateur|Elle pose le mouton près du pont.
-enfant-m|Merci.
-papa|Tu as accepté, Nino ?
-enfant-m|Oui, papa.
-maman|Bravo.
-narrateur|Le cheval finit le pont.
-narrateur|Il arrive de l'autre côté.
+papa|Tu le tiens, Nino ?
+enfant-m|Oui.
+narrateur|Les sabots tapent, puis se taisent.
+narrateur|Le cheval arrive de l'autre côté.
 enfant-m|Il est passé.
-copine|Le mouton aussi, après.
-papa|Clip, clop.
-enfant-m|Clip, clop.
-maman|Les gâteaux sont tièdes, maintenant.
-papa|On range le pont ?
+maman|Les gâteaux sont tièdes.
+papa|On plie le pont ?
 enfant-m|Oui.
 narrateur|Nino plie le carton.
-narrateur|Les lettres bleues se plient aussi.
-narrateur|Victorina pose le cheval.
-narrateur|Le mouton reste près d'elle.
-papa|Tu as fini le pont ?
-enfant-m|Oui, papa.</t>
+narrateur|Les lettres bleues se plient aussi.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>bois</t>
+          <t>cheval,carton</t>
         </is>
       </c>
     </row>
@@ -1978,17 +2038,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le cheval repose près du mouton. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. La farine dort encore sur les manches.</t>
+          <t>La plaque brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le bord. Nino pose le cheval près du mouton. On les garde près de nous ? Oui, maman. Ça sentait le beurre. Les gâteaux sont là. La plaque ne fume plus. Nino respire, plus large. On reste un peu ? Oui. Les joues de Nino se réchauffent. Le cheval reste tiède sous la main. Un éclat de plaque reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le cheval repose près du mouton. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. La farine dort encore sur les manches.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La plaque brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le bord. Nino pose le cheval près du mouton. On les garde près de nous ? Oui, maman. Ça sentait le beurre. Les gâteaux sont là. La plaque ne fume plus. Nino respire, plus large. On reste un peu ? Oui. Les joues de Nino se réchauffent. Le cheval reste tiède sous la main. Un &lt;emphasis level="moderate"&gt;éclat de plaque&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La plaque brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le bord. Nino pose le cheval près du mouton. On les garde près de nous ? Oui, maman. Ça sentait le beurre. Les gâteaux sont là. La plaque ne fume plus. Nino respire, plus large. On reste un peu ? Oui. Les joues de Nino se réchauffent. Le cheval reste tiède sous la main. Un &lt;emphasis&gt;éclat de plaque&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2035,7 +2095,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2043,10 +2103,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2055,12 +2115,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2069,17 +2129,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plaque</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2088,11 +2152,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2101,29 +2165,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_reste_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le cheval repose près du mouton.
-enfant-m|J'ai proposé.
-enfant-m|J'ai accepté.
-maman|Plusieurs réponses sont possibles.
-papa|Oui.
-narrateur|La farine dort encore sur les manches.</t>
+          <t>enfant-m|La plaque brillait, papa.
+papa|Tu le vois, comme tout à l'heure ?
+enfant-m|Oui, sur le bord.
+narrateur|Nino pose le cheval près du mouton.
+maman|On les garde près de nous ?
+enfant-m|Oui, maman.
+enfant-m|Ça sentait le beurre.
+maman|Les gâteaux sont là.
+narrateur|La plaque ne fume plus.
+narrateur|Nino respire, plus large.
+papa|On reste un peu ?
+enfant-m|Oui.
+narrateur|Les joues de Nino se réchauffent.
+narrateur|Le cheval reste tiède sous la main.
+narrateur|Un éclat de plaque reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>cuisine</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2222,6 +2304,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>